<commit_message>
current version of data, analyses optowell data
</commit_message>
<xml_diff>
--- a/26-07-23_optowell_test2/t12.xlsx
+++ b/26-07-23_optowell_test2/t12.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dungeon\Desktop\Yuhang\26-07-18 optowell exp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dungeon\Desktop\Yuhang\26-07-22 optowell exp 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5BDF9E0-52C5-49CF-9E5C-2CCA1DA3EACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC3AB333-55D7-4EE3-BAFE-DD8ABDA0FA65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{A89F5E0B-3C35-4FC0-BC07-F7DB8E98FF0B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{E265D536-B5C5-48B2-A005-6D7130A7BB6E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
     <author>dungeon</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{2AB1BB68-94A8-41E5-9522-C4907A8ECEF4}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{E01A6CC5-33E8-49E6-9712-C255BF109861}">
       <text>
         <r>
           <rPr>
@@ -110,7 +110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{467629DF-56A6-4282-8A3D-89D1295889EA}">
+    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{D2703B8A-488E-4741-A98E-D2B074B59285}">
       <text>
         <r>
           <rPr>
@@ -162,13 +162,13 @@
     <t>Date:</t>
   </si>
   <si>
-    <t>19/07/2026</t>
+    <t>22/07/2026</t>
   </si>
   <si>
     <t>Time:</t>
   </si>
   <si>
-    <t>02:00:01</t>
+    <t>23:33:27</t>
   </si>
   <si>
     <t>System</t>
@@ -222,10 +222,10 @@
     <t>Start Time:</t>
   </si>
   <si>
-    <t>19/07/2026 02:00:01</t>
-  </si>
-  <si>
-    <t>Temperature: 37.7 °C</t>
+    <t>22/07/2026 23:33:27</t>
+  </si>
+  <si>
+    <t>Temperature: 28.3 °C</t>
   </si>
   <si>
     <t>&lt;&gt;</t>
@@ -258,7 +258,7 @@
     <t>End Time:</t>
   </si>
   <si>
-    <t>19/07/2026 02:01:22</t>
+    <t>22/07/2026 23:34:49</t>
   </si>
   <si>
     <t>Label: GFP 395nm</t>
@@ -294,22 +294,22 @@
     <t>Lag Time</t>
   </si>
   <si>
-    <t>19/07/2026 02:01:25</t>
-  </si>
-  <si>
-    <t>Temperature: 37 °C</t>
-  </si>
-  <si>
-    <t>19/07/2026 02:02:43</t>
+    <t>22/07/2026 23:34:51</t>
+  </si>
+  <si>
+    <t>22/07/2026 23:36:09</t>
   </si>
   <si>
     <t>Label: GFP 480nm</t>
   </si>
   <si>
-    <t>19/07/2026 02:02:48</t>
-  </si>
-  <si>
-    <t>19/07/2026 02:04:05</t>
+    <t>22/07/2026 23:36:14</t>
+  </si>
+  <si>
+    <t>Temperature: 28.4 °C</t>
+  </si>
+  <si>
+    <t>22/07/2026 23:37:32</t>
   </si>
 </sst>
 </file>
@@ -482,13 +482,13 @@
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Tecan.At.Excel.Attenuation" xfId="6" xr:uid="{C44CE9AD-628D-4CE7-BCC3-A9D67DD421C4}"/>
-    <cellStyle name="Tecan.At.Excel.AutoGain_0" xfId="7" xr:uid="{BC080391-8C0F-473A-BBFC-05AD4F245459}"/>
-    <cellStyle name="Tecan.At.Excel.Error" xfId="1" xr:uid="{BF1E7292-73C8-4F31-8680-141206001068}"/>
-    <cellStyle name="Tecan.At.Excel.GFactorAndMeasurementBlank" xfId="5" xr:uid="{F4457023-163C-4BF3-ADEA-2183443E0514}"/>
-    <cellStyle name="Tecan.At.Excel.GFactorBlank" xfId="3" xr:uid="{ABCDDEDF-9A65-437F-8DD9-11998F023ED5}"/>
-    <cellStyle name="Tecan.At.Excel.GFactorReference" xfId="4" xr:uid="{8B79885D-DCE3-494D-9989-7E001DBE7E7F}"/>
-    <cellStyle name="Tecan.At.Excel.MeasurementBlank" xfId="2" xr:uid="{3B44A2E2-6D51-4039-83DC-30F78B27A1F6}"/>
+    <cellStyle name="Tecan.At.Excel.Attenuation" xfId="6" xr:uid="{FFFB5A06-6483-4127-B490-B58F347C7EB1}"/>
+    <cellStyle name="Tecan.At.Excel.AutoGain_0" xfId="7" xr:uid="{D6D2911A-A85E-4026-96DF-1E44DA0754FE}"/>
+    <cellStyle name="Tecan.At.Excel.Error" xfId="1" xr:uid="{547BB237-E723-4934-8F3C-923827CD77B9}"/>
+    <cellStyle name="Tecan.At.Excel.GFactorAndMeasurementBlank" xfId="5" xr:uid="{D56B9B1B-12A5-4DFB-97EA-68B3D1FA1F72}"/>
+    <cellStyle name="Tecan.At.Excel.GFactorBlank" xfId="3" xr:uid="{04EB5D3B-5371-49F9-A042-546163BAAE9A}"/>
+    <cellStyle name="Tecan.At.Excel.GFactorReference" xfId="4" xr:uid="{D73B0CEF-5C5C-4639-A961-1DCFD1D947CA}"/>
+    <cellStyle name="Tecan.At.Excel.MeasurementBlank" xfId="2" xr:uid="{6D93DE7E-B69A-40FB-B7C9-91791FE8C9AB}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -819,7 +819,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D9A5670-4838-4273-AE3E-4796566692D0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{597F907D-A7B1-47CA-BF6F-A0D162506A9F}">
   <dimension ref="A1:M101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1008,40 +1008,40 @@
         <v>31</v>
       </c>
       <c r="B25">
-        <v>0.24729999899864197</v>
+        <v>0.26339998841285706</v>
       </c>
       <c r="C25">
-        <v>0.26129999756813049</v>
+        <v>0.27320000529289246</v>
       </c>
       <c r="D25">
-        <v>0.26120001077651978</v>
+        <v>0.27309998869895935</v>
       </c>
       <c r="E25">
-        <v>0.15119999647140503</v>
+        <v>0.28650000691413879</v>
       </c>
       <c r="F25">
-        <v>0.28470000624656677</v>
+        <v>0.2824999988079071</v>
       </c>
       <c r="G25">
-        <v>0.29030001163482666</v>
+        <v>0.27720001339912415</v>
       </c>
       <c r="H25">
-        <v>0.29750001430511475</v>
+        <v>0.27939999103546143</v>
       </c>
       <c r="I25">
-        <v>0.27669999003410339</v>
+        <v>0.2418999969959259</v>
       </c>
       <c r="J25">
-        <v>0.27529999613761902</v>
+        <v>0.25909999012947083</v>
       </c>
       <c r="K25">
-        <v>0.28600001335144043</v>
+        <v>0.35809999704360962</v>
       </c>
       <c r="L25">
-        <v>0.28619998693466187</v>
+        <v>0.3783000111579895</v>
       </c>
       <c r="M25">
-        <v>0.28700000047683716</v>
+        <v>0.37259998917579651</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
@@ -1049,40 +1049,40 @@
         <v>32</v>
       </c>
       <c r="B26">
-        <v>0.14880000054836273</v>
+        <v>0.13050000369548798</v>
       </c>
       <c r="C26">
-        <v>0.15469999611377716</v>
+        <v>0.12349999696016312</v>
       </c>
       <c r="D26">
-        <v>0.14259999990463257</v>
+        <v>0.13789999485015869</v>
       </c>
       <c r="E26">
-        <v>0.14509999752044678</v>
+        <v>0.13249999284744263</v>
       </c>
       <c r="F26">
-        <v>0.13969999551773071</v>
+        <v>0.13539999723434448</v>
       </c>
       <c r="G26">
-        <v>0.1500999927520752</v>
+        <v>0.14460000395774841</v>
       </c>
       <c r="H26">
-        <v>0.23459999263286591</v>
+        <v>0.19869999587535858</v>
       </c>
       <c r="I26">
-        <v>0.18479999899864197</v>
+        <v>0.18979999423027039</v>
       </c>
       <c r="J26">
-        <v>0.17739999294281006</v>
+        <v>0.19449999928474426</v>
       </c>
       <c r="K26">
-        <v>0.28290000557899475</v>
+        <v>0.36239999532699585</v>
       </c>
       <c r="L26">
-        <v>0.29229998588562012</v>
+        <v>0.36269998550415039</v>
       </c>
       <c r="M26">
-        <v>0.28319999575614929</v>
+        <v>0.36750000715255737</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
@@ -1090,40 +1090,40 @@
         <v>33</v>
       </c>
       <c r="B27">
-        <v>0.13779999315738678</v>
+        <v>0.11580000072717667</v>
       </c>
       <c r="C27">
-        <v>0.13480000197887421</v>
+        <v>0.12200000137090683</v>
       </c>
       <c r="D27">
-        <v>0.13349999487400055</v>
+        <v>0.12330000102519989</v>
       </c>
       <c r="E27">
-        <v>0.13189999759197235</v>
+        <v>0.12700000405311584</v>
       </c>
       <c r="F27">
-        <v>0.13230000436306</v>
+        <v>0.12849999964237213</v>
       </c>
       <c r="G27">
-        <v>0.1307000070810318</v>
+        <v>0.12770000100135803</v>
       </c>
       <c r="H27">
-        <v>0.17059999704360962</v>
+        <v>0.18269999325275421</v>
       </c>
       <c r="I27">
-        <v>0.16570000350475311</v>
+        <v>0.1785999983549118</v>
       </c>
       <c r="J27">
-        <v>0.16599999368190765</v>
+        <v>0.1867000013589859</v>
       </c>
       <c r="K27">
-        <v>0.29530000686645508</v>
+        <v>0.35859999060630798</v>
       </c>
       <c r="L27">
-        <v>0.28799998760223389</v>
+        <v>0.3578999936580658</v>
       </c>
       <c r="M27">
-        <v>0.2856999933719635</v>
+        <v>0.38339999318122864</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
@@ -1131,40 +1131,40 @@
         <v>34</v>
       </c>
       <c r="B28">
-        <v>0.21240000426769257</v>
+        <v>0.23610000312328339</v>
       </c>
       <c r="C28">
-        <v>0.2151000052690506</v>
+        <v>0.18950000405311584</v>
       </c>
       <c r="D28">
-        <v>0.2207999974489212</v>
+        <v>0.25429999828338623</v>
       </c>
       <c r="E28">
-        <v>0.21070000529289246</v>
+        <v>0.27649998664855957</v>
       </c>
       <c r="F28">
-        <v>0.22259999811649323</v>
+        <v>0.27169999480247498</v>
       </c>
       <c r="G28">
-        <v>0.24699999392032623</v>
+        <v>0.29879999160766602</v>
       </c>
       <c r="H28">
-        <v>0.3010999858379364</v>
+        <v>0.49210000038146973</v>
       </c>
       <c r="I28">
-        <v>0.1729000061750412</v>
+        <v>0.17550000548362732</v>
       </c>
       <c r="J28">
-        <v>0.17180000245571136</v>
+        <v>0.1906999945640564</v>
       </c>
       <c r="K28">
-        <v>0.32179999351501465</v>
+        <v>0.34110000729560852</v>
       </c>
       <c r="L28">
-        <v>0.30340000987052917</v>
+        <v>0.36219999194145203</v>
       </c>
       <c r="M28">
-        <v>0.29750001430511475</v>
+        <v>0.36680001020431519</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
@@ -1172,40 +1172,40 @@
         <v>35</v>
       </c>
       <c r="B29">
-        <v>0.27140000462532043</v>
+        <v>0.30680000782012939</v>
       </c>
       <c r="C29">
-        <v>0.27990001440048218</v>
+        <v>0.31799998879432678</v>
       </c>
       <c r="D29">
-        <v>0.28909999132156372</v>
+        <v>0.32910001277923584</v>
       </c>
       <c r="E29">
-        <v>0.30550000071525574</v>
+        <v>0.33100000023841858</v>
       </c>
       <c r="F29">
-        <v>0.30579999089241028</v>
+        <v>0.32929998636245728</v>
       </c>
       <c r="G29">
-        <v>0.31270000338554382</v>
+        <v>0.36329999566078186</v>
       </c>
       <c r="H29">
-        <v>0.31889998912811279</v>
+        <v>0.48059999942779541</v>
       </c>
       <c r="I29">
-        <v>0.30070000886917114</v>
+        <v>0.33390000462532043</v>
       </c>
       <c r="J29">
-        <v>0.28060001134872437</v>
+        <v>0.2630000114440918</v>
       </c>
       <c r="K29">
-        <v>0.30050000548362732</v>
+        <v>0.35530000925064087</v>
       </c>
       <c r="L29">
-        <v>0.29800000786781311</v>
+        <v>0.35989999771118164</v>
       </c>
       <c r="M29">
-        <v>0.30169999599456787</v>
+        <v>0.37529999017715454</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
@@ -1213,40 +1213,40 @@
         <v>36</v>
       </c>
       <c r="B30">
-        <v>0.27419999241828918</v>
+        <v>0.35359999537467957</v>
       </c>
       <c r="C30">
-        <v>0.30689999461174011</v>
+        <v>0.35240000486373901</v>
       </c>
       <c r="D30">
-        <v>0.30309998989105225</v>
+        <v>0.3409000039100647</v>
       </c>
       <c r="E30">
-        <v>0.30349999666213989</v>
+        <v>0.35060000419616699</v>
       </c>
       <c r="F30">
-        <v>0.30390000343322754</v>
+        <v>0.34520000219345093</v>
       </c>
       <c r="G30">
-        <v>0.30899998545646667</v>
+        <v>0.35229998826980591</v>
       </c>
       <c r="H30">
-        <v>0.31340000033378601</v>
+        <v>0.33860000967979431</v>
       </c>
       <c r="I30">
-        <v>0.30950000882148743</v>
+        <v>0.34720000624656677</v>
       </c>
       <c r="J30">
-        <v>0.31499999761581421</v>
+        <v>0.31940001249313354</v>
       </c>
       <c r="K30">
-        <v>0.30410000681877136</v>
+        <v>0.3580000102519989</v>
       </c>
       <c r="L30">
-        <v>0.2939000129699707</v>
+        <v>0.37839999794960022</v>
       </c>
       <c r="M30">
-        <v>0.30849999189376831</v>
+        <v>0.37209999561309814</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
@@ -1254,40 +1254,40 @@
         <v>37</v>
       </c>
       <c r="B31">
-        <v>0.29989999532699585</v>
+        <v>0.36239999532699585</v>
       </c>
       <c r="C31">
-        <v>0.31560000777244568</v>
+        <v>0.36640000343322754</v>
       </c>
       <c r="D31">
-        <v>0.29940000176429749</v>
+        <v>0.37529999017715454</v>
       </c>
       <c r="E31">
-        <v>0.30910000205039978</v>
+        <v>0.38499999046325684</v>
       </c>
       <c r="F31">
-        <v>0.30460000038146973</v>
+        <v>0.383899986743927</v>
       </c>
       <c r="G31">
-        <v>0.31310001015663147</v>
+        <v>0.38760000467300415</v>
       </c>
       <c r="H31">
-        <v>0.31380000710487366</v>
+        <v>0.36970001459121704</v>
       </c>
       <c r="I31">
-        <v>0.30050000548362732</v>
+        <v>0.34279999136924744</v>
       </c>
       <c r="J31">
-        <v>0.30889999866485596</v>
+        <v>0.31499999761581421</v>
       </c>
       <c r="K31">
-        <v>0.30849999189376831</v>
+        <v>0.37299999594688416</v>
       </c>
       <c r="L31">
-        <v>0.29739999771118164</v>
+        <v>0.3781999945640564</v>
       </c>
       <c r="M31">
-        <v>0.29679998755455017</v>
+        <v>0.37569999694824219</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
@@ -1295,40 +1295,40 @@
         <v>38</v>
       </c>
       <c r="B32">
-        <v>0.28159999847412109</v>
+        <v>0.34509998559951782</v>
       </c>
       <c r="C32">
-        <v>0.32429999113082886</v>
+        <v>0.36809998750686646</v>
       </c>
       <c r="D32">
-        <v>0.31349998712539673</v>
+        <v>0.36529999971389771</v>
       </c>
       <c r="E32">
-        <v>0.30059999227523804</v>
+        <v>0.39789998531341553</v>
       </c>
       <c r="F32">
-        <v>0.30320000648498535</v>
+        <v>0.4018000066280365</v>
       </c>
       <c r="G32">
-        <v>0.3140999972820282</v>
+        <v>0.40290001034736633</v>
       </c>
       <c r="H32">
-        <v>0.30219998955726624</v>
+        <v>0.37110000848770142</v>
       </c>
       <c r="I32">
-        <v>0.28929999470710754</v>
+        <v>0.3474000096321106</v>
       </c>
       <c r="J32">
-        <v>0.30370000004768372</v>
+        <v>0.3246999979019165</v>
       </c>
       <c r="K32">
-        <v>0.30640000104904175</v>
+        <v>0.3718000054359436</v>
       </c>
       <c r="L32">
-        <v>0.29580000042915344</v>
+        <v>0.37360000610351563</v>
       </c>
       <c r="M32">
-        <v>0.29809999465942383</v>
+        <v>0.37770000100135803</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -1458,7 +1458,7 @@
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.25">
@@ -1507,40 +1507,40 @@
         <v>31</v>
       </c>
       <c r="B57">
-        <v>1926</v>
+        <v>821</v>
       </c>
       <c r="C57">
-        <v>2231</v>
+        <v>852</v>
       </c>
       <c r="D57">
-        <v>2206</v>
+        <v>815</v>
       </c>
       <c r="E57">
-        <v>274</v>
+        <v>594</v>
       </c>
       <c r="F57">
-        <v>2021</v>
+        <v>530</v>
       </c>
       <c r="G57">
-        <v>2185</v>
+        <v>610</v>
       </c>
       <c r="H57">
-        <v>793</v>
+        <v>620</v>
       </c>
       <c r="I57">
-        <v>462</v>
+        <v>455</v>
       </c>
       <c r="J57">
-        <v>462</v>
+        <v>542</v>
       </c>
       <c r="K57">
-        <v>537</v>
+        <v>774</v>
       </c>
       <c r="L57">
-        <v>526</v>
+        <v>970</v>
       </c>
       <c r="M57">
-        <v>439</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
@@ -1548,40 +1548,40 @@
         <v>32</v>
       </c>
       <c r="B58">
-        <v>143</v>
+        <v>68</v>
       </c>
       <c r="C58">
-        <v>141</v>
+        <v>56</v>
       </c>
       <c r="D58">
-        <v>125</v>
+        <v>65</v>
       </c>
       <c r="E58">
-        <v>135</v>
+        <v>62</v>
       </c>
       <c r="F58">
-        <v>131</v>
+        <v>69</v>
       </c>
       <c r="G58">
-        <v>150</v>
+        <v>76</v>
       </c>
       <c r="H58">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="I58">
-        <v>174</v>
+        <v>233</v>
       </c>
       <c r="J58">
-        <v>137</v>
+        <v>272</v>
       </c>
       <c r="K58">
-        <v>285</v>
+        <v>514</v>
       </c>
       <c r="L58">
-        <v>283</v>
+        <v>627</v>
       </c>
       <c r="M58">
-        <v>282</v>
+        <v>781</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.25">
@@ -1589,40 +1589,40 @@
         <v>33</v>
       </c>
       <c r="B59">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="C59">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="D59">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="E59">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="F59">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="G59">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="H59">
-        <v>122</v>
+        <v>183</v>
       </c>
       <c r="I59">
-        <v>104</v>
+        <v>162</v>
       </c>
       <c r="J59">
-        <v>119</v>
+        <v>186</v>
       </c>
       <c r="K59">
-        <v>228</v>
+        <v>411</v>
       </c>
       <c r="L59">
-        <v>218</v>
+        <v>490</v>
       </c>
       <c r="M59">
-        <v>201</v>
+        <v>679</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.25">
@@ -1630,40 +1630,40 @@
         <v>34</v>
       </c>
       <c r="B60">
+        <v>2044</v>
+      </c>
+      <c r="C60">
+        <v>831</v>
+      </c>
+      <c r="D60">
+        <v>1594</v>
+      </c>
+      <c r="E60">
         <v>1431</v>
       </c>
-      <c r="C60">
-        <v>1541</v>
-      </c>
-      <c r="D60">
-        <v>1584</v>
-      </c>
-      <c r="E60">
-        <v>984</v>
-      </c>
       <c r="F60">
-        <v>1136</v>
+        <v>1233</v>
       </c>
       <c r="G60">
-        <v>1561</v>
+        <v>1530</v>
       </c>
       <c r="H60">
-        <v>2575</v>
+        <v>732</v>
       </c>
       <c r="I60">
-        <v>114</v>
+        <v>157</v>
       </c>
       <c r="J60">
-        <v>116</v>
+        <v>180</v>
       </c>
       <c r="K60">
-        <v>210</v>
+        <v>374</v>
       </c>
       <c r="L60">
-        <v>214</v>
+        <v>471</v>
       </c>
       <c r="M60">
-        <v>203</v>
+        <v>640</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.25">
@@ -1671,40 +1671,40 @@
         <v>35</v>
       </c>
       <c r="B61">
-        <v>2794</v>
+        <v>3033</v>
       </c>
       <c r="C61">
-        <v>3278</v>
+        <v>2851</v>
       </c>
       <c r="D61">
-        <v>3298</v>
+        <v>2622</v>
       </c>
       <c r="E61">
-        <v>3165</v>
+        <v>1962</v>
       </c>
       <c r="F61">
-        <v>3137</v>
+        <v>1899</v>
       </c>
       <c r="G61">
-        <v>3157</v>
+        <v>2146</v>
       </c>
       <c r="H61">
-        <v>4337</v>
+        <v>2982</v>
       </c>
       <c r="I61">
-        <v>1440</v>
+        <v>929</v>
       </c>
       <c r="J61">
-        <v>389</v>
+        <v>440</v>
       </c>
       <c r="K61">
-        <v>260</v>
+        <v>461</v>
       </c>
       <c r="L61">
-        <v>240</v>
+        <v>563</v>
       </c>
       <c r="M61">
-        <v>223</v>
+        <v>767</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
@@ -1712,40 +1712,40 @@
         <v>36</v>
       </c>
       <c r="B62">
-        <v>2827</v>
+        <v>4461</v>
       </c>
       <c r="C62">
-        <v>3651</v>
+        <v>3653</v>
       </c>
       <c r="D62">
-        <v>3536</v>
+        <v>2972</v>
       </c>
       <c r="E62">
-        <v>3104</v>
+        <v>2556</v>
       </c>
       <c r="F62">
-        <v>3079</v>
+        <v>2316</v>
       </c>
       <c r="G62">
-        <v>3099</v>
+        <v>2519</v>
       </c>
       <c r="H62">
-        <v>4325</v>
+        <v>3604</v>
       </c>
       <c r="I62">
-        <v>2466</v>
+        <v>1870</v>
       </c>
       <c r="J62">
-        <v>609</v>
+        <v>886</v>
       </c>
       <c r="K62">
-        <v>303</v>
+        <v>610</v>
       </c>
       <c r="L62">
-        <v>246</v>
+        <v>710</v>
       </c>
       <c r="M62">
-        <v>321</v>
+        <v>868</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
@@ -1753,40 +1753,40 @@
         <v>37</v>
       </c>
       <c r="B63">
-        <v>3475</v>
+        <v>6983</v>
       </c>
       <c r="C63">
-        <v>4112</v>
+        <v>6013</v>
       </c>
       <c r="D63">
-        <v>3870</v>
+        <v>5766</v>
       </c>
       <c r="E63">
-        <v>3488</v>
+        <v>4917</v>
       </c>
       <c r="F63">
-        <v>3461</v>
+        <v>4783</v>
       </c>
       <c r="G63">
-        <v>3546</v>
+        <v>4721</v>
       </c>
       <c r="H63">
-        <v>4240</v>
+        <v>4279</v>
       </c>
       <c r="I63">
-        <v>1476</v>
+        <v>1415</v>
       </c>
       <c r="J63">
-        <v>576</v>
+        <v>920</v>
       </c>
       <c r="K63">
-        <v>293</v>
+        <v>768</v>
       </c>
       <c r="L63">
-        <v>271</v>
+        <v>860</v>
       </c>
       <c r="M63">
-        <v>226</v>
+        <v>947</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.25">
@@ -1794,40 +1794,40 @@
         <v>38</v>
       </c>
       <c r="B64">
-        <v>3298</v>
+        <v>6922</v>
       </c>
       <c r="C64">
-        <v>4113</v>
+        <v>6353</v>
       </c>
       <c r="D64">
-        <v>3730</v>
+        <v>5403</v>
       </c>
       <c r="E64">
-        <v>3180</v>
+        <v>5139</v>
       </c>
       <c r="F64">
-        <v>3165</v>
+        <v>5036</v>
       </c>
       <c r="G64">
-        <v>3356</v>
+        <v>4985</v>
       </c>
       <c r="H64">
-        <v>3693</v>
+        <v>3984</v>
       </c>
       <c r="I64">
-        <v>738</v>
+        <v>1257</v>
       </c>
       <c r="J64">
-        <v>486</v>
+        <v>956</v>
       </c>
       <c r="K64">
-        <v>282</v>
+        <v>971</v>
       </c>
       <c r="L64">
-        <v>244</v>
+        <v>950</v>
       </c>
       <c r="M64">
-        <v>227</v>
+        <v>973</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -1835,12 +1835,12 @@
         <v>39</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -1952,12 +1952,12 @@
         <v>27</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.25">
@@ -2006,40 +2006,40 @@
         <v>31</v>
       </c>
       <c r="B89">
-        <v>1996</v>
+        <v>811</v>
       </c>
       <c r="C89">
-        <v>2305</v>
+        <v>862</v>
       </c>
       <c r="D89">
-        <v>2281</v>
+        <v>808</v>
       </c>
       <c r="E89">
-        <v>254</v>
+        <v>570</v>
       </c>
       <c r="F89">
-        <v>2018</v>
+        <v>498</v>
       </c>
       <c r="G89">
-        <v>2156</v>
+        <v>582</v>
       </c>
       <c r="H89">
-        <v>756</v>
+        <v>495</v>
       </c>
       <c r="I89">
-        <v>426</v>
+        <v>355</v>
       </c>
       <c r="J89">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="K89">
-        <v>463</v>
+        <v>647</v>
       </c>
       <c r="L89">
-        <v>448</v>
+        <v>870</v>
       </c>
       <c r="M89">
-        <v>361</v>
+        <v>977</v>
       </c>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.25">
@@ -2047,40 +2047,40 @@
         <v>32</v>
       </c>
       <c r="B90">
-        <v>115</v>
+        <v>48</v>
       </c>
       <c r="C90">
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="D90">
-        <v>93</v>
+        <v>45</v>
       </c>
       <c r="E90">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="F90">
-        <v>104</v>
+        <v>52</v>
       </c>
       <c r="G90">
-        <v>122</v>
+        <v>55</v>
       </c>
       <c r="H90">
-        <v>198</v>
+        <v>149</v>
       </c>
       <c r="I90">
-        <v>70</v>
+        <v>133</v>
       </c>
       <c r="J90">
-        <v>61</v>
+        <v>171</v>
       </c>
       <c r="K90">
-        <v>209</v>
+        <v>385</v>
       </c>
       <c r="L90">
-        <v>212</v>
+        <v>516</v>
       </c>
       <c r="M90">
-        <v>185</v>
+        <v>689</v>
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.25">
@@ -2088,40 +2088,40 @@
         <v>33</v>
       </c>
       <c r="B91">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C91">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D91">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="E91">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="F91">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="G91">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="H91">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="I91">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="J91">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="K91">
-        <v>139</v>
+        <v>283</v>
       </c>
       <c r="L91">
-        <v>148</v>
+        <v>369</v>
       </c>
       <c r="M91">
-        <v>133</v>
+        <v>586</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.25">
@@ -2129,40 +2129,40 @@
         <v>34</v>
       </c>
       <c r="B92">
-        <v>1439</v>
+        <v>2088</v>
       </c>
       <c r="C92">
-        <v>1515</v>
+        <v>841</v>
       </c>
       <c r="D92">
-        <v>1605</v>
+        <v>1623</v>
       </c>
       <c r="E92">
-        <v>948</v>
+        <v>1460</v>
       </c>
       <c r="F92">
-        <v>1102</v>
+        <v>1281</v>
       </c>
       <c r="G92">
-        <v>1586</v>
+        <v>1570</v>
       </c>
       <c r="H92">
-        <v>2545</v>
+        <v>677</v>
       </c>
       <c r="I92">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="J92">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="K92">
-        <v>133</v>
+        <v>253</v>
       </c>
       <c r="L92">
-        <v>138</v>
+        <v>354</v>
       </c>
       <c r="M92">
-        <v>135</v>
+        <v>547</v>
       </c>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.25">
@@ -2170,40 +2170,40 @@
         <v>35</v>
       </c>
       <c r="B93">
-        <v>2866</v>
+        <v>3086</v>
       </c>
       <c r="C93">
-        <v>3399</v>
+        <v>2884</v>
       </c>
       <c r="D93">
-        <v>3434</v>
+        <v>2679</v>
       </c>
       <c r="E93">
-        <v>2974</v>
+        <v>1908</v>
       </c>
       <c r="F93">
-        <v>2945</v>
+        <v>1823</v>
       </c>
       <c r="G93">
-        <v>2969</v>
+        <v>2070</v>
       </c>
       <c r="H93">
-        <v>4243</v>
+        <v>3072</v>
       </c>
       <c r="I93">
-        <v>1424</v>
+        <v>857</v>
       </c>
       <c r="J93">
-        <v>351</v>
+        <v>368</v>
       </c>
       <c r="K93">
-        <v>190</v>
+        <v>341</v>
       </c>
       <c r="L93">
-        <v>164</v>
+        <v>461</v>
       </c>
       <c r="M93">
-        <v>143</v>
+        <v>679</v>
       </c>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.25">
@@ -2211,40 +2211,40 @@
         <v>36</v>
       </c>
       <c r="B94">
-        <v>2917</v>
+        <v>4463</v>
       </c>
       <c r="C94">
-        <v>3755</v>
+        <v>3667</v>
       </c>
       <c r="D94">
-        <v>3638</v>
+        <v>2974</v>
       </c>
       <c r="E94">
-        <v>2878</v>
+        <v>2434</v>
       </c>
       <c r="F94">
-        <v>2858</v>
+        <v>2236</v>
       </c>
       <c r="G94">
-        <v>2860</v>
+        <v>2403</v>
       </c>
       <c r="H94">
-        <v>4209</v>
+        <v>3588</v>
       </c>
       <c r="I94">
-        <v>2441</v>
+        <v>1617</v>
       </c>
       <c r="J94">
-        <v>555</v>
+        <v>827</v>
       </c>
       <c r="K94">
-        <v>235</v>
+        <v>499</v>
       </c>
       <c r="L94">
-        <v>183</v>
+        <v>622</v>
       </c>
       <c r="M94">
-        <v>147</v>
+        <v>784</v>
       </c>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.25">
@@ -2252,40 +2252,40 @@
         <v>37</v>
       </c>
       <c r="B95">
-        <v>3545</v>
+        <v>6710</v>
       </c>
       <c r="C95">
-        <v>3968</v>
+        <v>5750</v>
       </c>
       <c r="D95">
-        <v>3813</v>
+        <v>5461</v>
       </c>
       <c r="E95">
-        <v>3180</v>
+        <v>4672</v>
       </c>
       <c r="F95">
-        <v>3186</v>
+        <v>4529</v>
       </c>
       <c r="G95">
-        <v>3256</v>
+        <v>4474</v>
       </c>
       <c r="H95">
-        <v>4113</v>
+        <v>4112</v>
       </c>
       <c r="I95">
-        <v>1431</v>
+        <v>1314</v>
       </c>
       <c r="J95">
-        <v>508</v>
+        <v>865</v>
       </c>
       <c r="K95">
-        <v>223</v>
+        <v>651</v>
       </c>
       <c r="L95">
-        <v>185</v>
+        <v>767</v>
       </c>
       <c r="M95">
-        <v>158</v>
+        <v>856</v>
       </c>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.25">
@@ -2293,40 +2293,40 @@
         <v>38</v>
       </c>
       <c r="B96">
-        <v>3393</v>
+        <v>6669</v>
       </c>
       <c r="C96">
-        <v>3962</v>
+        <v>6125</v>
       </c>
       <c r="D96">
-        <v>3617</v>
+        <v>5122</v>
       </c>
       <c r="E96">
-        <v>2936</v>
+        <v>4873</v>
       </c>
       <c r="F96">
-        <v>2951</v>
+        <v>4783</v>
       </c>
       <c r="G96">
-        <v>3131</v>
+        <v>4656</v>
       </c>
       <c r="H96">
-        <v>3578</v>
+        <v>3746</v>
       </c>
       <c r="I96">
-        <v>678</v>
+        <v>1160</v>
       </c>
       <c r="J96">
-        <v>428</v>
+        <v>901</v>
       </c>
       <c r="K96">
-        <v>205</v>
+        <v>874</v>
       </c>
       <c r="L96">
-        <v>177</v>
+        <v>874</v>
       </c>
       <c r="M96">
-        <v>153</v>
+        <v>877</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
@@ -2344,7 +2344,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF333A3D-B800-433B-9B71-C261B3B60D2F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D5F3618-4D11-46D9-A7DB-F1818C67DD48}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>